<commit_message>
Update Sehore LULC Area Statistics file with new data
</commit_message>
<xml_diff>
--- a/Sehore_Data_and_Pridictions_CSVs/Sehore_LULC_Area_Statistics_2017_2020.xlsx
+++ b/Sehore_Data_and_Pridictions_CSVs/Sehore_LULC_Area_Statistics_2017_2020.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Epics\SehoreDataandPridictionsCSVs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Epics\Sehore_Data_and_Pridictions_CSVs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C67E30DA-FCF1-4247-B819-54B5F03EDF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9607E6AD-3929-4C6B-99D6-71915857F859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,9 +201,6 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -224,6 +221,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -508,7 +508,7 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="21.33203125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
@@ -516,207 +516,207 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>25.42</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>42.2</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <f t="shared" ref="E2:E8" si="0">D2-C2</f>
         <v>16.78</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <f t="shared" ref="F2:F8" si="1">IF(C2=0,"",(D2-C2)/C2*100)</f>
         <v>66.01101494885917</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>897.01</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>640.86</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f t="shared" si="0"/>
         <v>-256.14999999999998</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <f t="shared" si="1"/>
         <v>-28.555980423852574</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>0.46</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>0.69</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f t="shared" si="0"/>
         <v>0.22999999999999993</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <f t="shared" si="1"/>
         <v>49.999999999999986</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>5590.13</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>5828.81</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <f t="shared" si="0"/>
         <v>238.68000000000029</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <f t="shared" si="1"/>
         <v>4.2696681472523945</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>33.01</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>33.700000000000003</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
         <v>0.69000000000000483</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <f t="shared" si="1"/>
         <v>2.0902756740381849</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>7</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>0.42</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>0.19</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <f t="shared" si="0"/>
         <v>-0.22999999999999998</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <f t="shared" si="1"/>
         <v>-54.761904761904759</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>1.6</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>1.6</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <f>SUM(C2:C8)</f>
         <v>6548.0500000000011</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <f>SUM(D2:D8)</f>
         <v>6548.05</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <f>SUM(E2:E8)</f>
         <v>3.0953017926549364E-13</v>
       </c>
-      <c r="F9" s="8"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="11" spans="1:6" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>